<commit_message>
Update Skeena steelhead to include 2025 numbers from Tyee
</commit_message>
<xml_diff>
--- a/data/data-sources_2026.xlsx
+++ b/data/data-sources_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hhunter\Documents\state-of-salmon\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Documents/2_PSF/GitHub/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BADB120-6245-4042-9856-A9E91FD8CA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1DE3D1-D305-DC41-BEFF-E212F7E53FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15525" yWindow="-18120" windowWidth="25440" windowHeight="15270" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,6 +40,7 @@
   <authors>
     <author>tc={303AFB4F-4F8A-4CA2-B10F-5008E0D1F507}</author>
     <author>tc={B95E03CA-958C-46CF-B95C-F5F3C9D83C4F}</author>
+    <author>tc={C3CEA22A-2BE0-AA4B-8455-9328949CA654}</author>
   </authors>
   <commentList>
     <comment ref="B16" authorId="0" shapeId="0" xr:uid="{303AFB4F-4F8A-4CA2-B10F-5008E0D1F507}">
@@ -58,12 +59,20 @@
     Need date and source </t>
       </text>
     </comment>
+    <comment ref="B27" authorId="2" shapeId="0" xr:uid="{C3CEA22A-2BE0-AA4B-8455-9328949CA654}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Used for 2025 source only; past years from ProvBC_20240929</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>source_id</t>
   </si>
@@ -261,6 +270,12 @@
   </si>
   <si>
     <t>DFO. 2025. West Coast of Vancouver Island Stock Assessment October 24, 2025: Escapement Bulletin #7 - all salmon species. Produced by DFO South Coast Stock Assessment and provided to Pacific Salmon Foundation by Diana McHugh on October 24, 2025.</t>
+  </si>
+  <si>
+    <t>Ramsay_20250814</t>
+  </si>
+  <si>
+    <t>Ramsay, M. 2025. Skeena Steelhead Recreational Fishery Update – 2025 Season. Ministry of Water, Land and Resource Stewardship, Victoria, B.C. Available from https://www2.gov.bc.ca/assets/gov/sports-recreation-arts-and-culture/outdoor-recreation/fishing-and-hunting/freshwater-fishing/skeena_steelhead_update_august_14_2025.pdf [accessed 13 April 2026].</t>
   </si>
 </sst>
 </file>
@@ -310,13 +325,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -335,6 +350,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -349,7 +370,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -375,6 +396,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -396,6 +421,7 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Hannah Hunter" id="{7D08CB21-0BF6-43C4-A3F6-F3C5403704B3}" userId="S::hhunter@psf.ca::162a122b-3bef-442e-baaa-85158fe52bc1" providerId="AD"/>
+  <person displayName="Stephanie Peacock" id="{510EDA56-7C0E-2341-A6E6-B2F29D200F02}" userId="S::speacock@psf.ca::bf4adfa3-bca4-4097-88ce-f14a2b5bdd2c" providerId="AD"/>
 </personList>
 </file>
 
@@ -722,19 +748,22 @@
   <threadedComment ref="B17" dT="2026-04-09T17:46:27.74" personId="{7D08CB21-0BF6-43C4-A3F6-F3C5403704B3}" id="{B95E03CA-958C-46CF-B95C-F5F3C9D83C4F}">
     <text xml:space="preserve">Need date and source </text>
   </threadedComment>
+  <threadedComment ref="B27" dT="2026-04-13T19:13:48.42" personId="{510EDA56-7C0E-2341-A6E6-B2F29D200F02}" id="{C3CEA22A-2BE0-AA4B-8455-9328949CA654}">
+    <text>Used for 2025 source only; past years from ProvBC_20240929</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24029AEC-6FE5-6340-8374-FCF69BAFD37B}">
-  <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.69921875" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
     <col min="2" max="2" width="127" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -742,7 +771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -751,7 +780,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -759,7 +788,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -767,7 +796,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -775,7 +804,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -783,7 +812,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -791,7 +820,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -799,7 +828,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -807,7 +836,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -815,7 +844,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="68" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -823,7 +852,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -831,7 +860,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -839,7 +868,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -847,7 +876,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>46</v>
       </c>
@@ -855,7 +884,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>50</v>
       </c>
@@ -863,7 +892,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>49</v>
       </c>
@@ -871,7 +900,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -879,7 +908,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="51" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -887,7 +916,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -895,7 +924,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -903,7 +932,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -911,7 +940,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -919,7 +948,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -927,7 +956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -935,12 +964,20 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>12</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Skeena steelhead data to reflect Sept 2 2025 estimate shared via email
</commit_message>
<xml_diff>
--- a/data/data-sources_2026.xlsx
+++ b/data/data-sources_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Documents/2_PSF/GitHub/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1DE3D1-D305-DC41-BEFF-E212F7E53FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180B61AA-B4B2-3540-98A5-110C3A707260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>source_id</t>
   </si>
@@ -276,6 +276,12 @@
   </si>
   <si>
     <t>Ramsay, M. 2025. Skeena Steelhead Recreational Fishery Update – 2025 Season. Ministry of Water, Land and Resource Stewardship, Victoria, B.C. Available from https://www2.gov.bc.ca/assets/gov/sports-recreation-arts-and-culture/outdoor-recreation/fishing-and-hunting/freshwater-fishing/skeena_steelhead_update_august_14_2025.pdf [accessed 13 April 2026].</t>
+  </si>
+  <si>
+    <t>Province of British Columbia. 2023. Estimated Escapement of Skeena Summer Steelhead at the Tyee Test Fishery, 1956 - 2024 - All Years to Sept 2, 2025. Provided to Pacific Salmon Foundation by Kenji Miyazaki on September 3, 2025.</t>
+  </si>
+  <si>
+    <t>ProvBC_20250903</t>
   </si>
 </sst>
 </file>
@@ -325,10 +331,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Tahoma"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -370,7 +377,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -398,6 +405,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -756,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24029AEC-6FE5-6340-8374-FCF69BAFD37B}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -980,6 +990,14 @@
         <v>53</v>
       </c>
     </row>
+    <row r="28" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B26">
     <sortCondition ref="A1:A26"/>

</xml_diff>

<commit_message>
added Yakoun Chinook data (spawners only) and updated data sources
</commit_message>
<xml_diff>
--- a/data/data-sources_2026.xlsx
+++ b/data/data-sources_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Documents/2_PSF/GitHub/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180B61AA-B4B2-3540-98A5-110C3A707260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91F8EC7-DF9C-E34A-8FC9-4CC78378100C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>source_id</t>
   </si>
@@ -282,6 +282,12 @@
   </si>
   <si>
     <t>ProvBC_20250903</t>
+  </si>
+  <si>
+    <t>Spoljaric_20260409</t>
+  </si>
+  <si>
+    <t>Spoljaric, Mark. 2026. Summary of Yakoun Chinook escapement estimates, 2021 - 2025. Provided to Pacific Salmon Foundation by Mark Spoljaric (Haida Fisheries Program) on April 9, 2026.</t>
   </si>
 </sst>
 </file>
@@ -766,7 +772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24029AEC-6FE5-6340-8374-FCF69BAFD37B}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -998,6 +1004,14 @@
         <v>54</v>
       </c>
     </row>
+    <row r="29" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B26">
     <sortCondition ref="A1:A26"/>

</xml_diff>

<commit_message>
Fraser pink and Fraser sockeye data updated from PSC; 2025 data files moved to Dropbox archive and data-sources_2026 updated with source_id = PSC_20260417
</commit_message>
<xml_diff>
--- a/data/data-sources_2026.xlsx
+++ b/data/data-sources_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Documents/2_PSF/GitHub/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91F8EC7-DF9C-E34A-8FC9-4CC78378100C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4CF1B79-3298-D141-82DA-895478F74096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>source_id</t>
   </si>
@@ -288,6 +288,12 @@
   </si>
   <si>
     <t>Spoljaric, Mark. 2026. Summary of Yakoun Chinook escapement estimates, 2021 - 2025. Provided to Pacific Salmon Foundation by Mark Spoljaric (Haida Fisheries Program) on April 9, 2026.</t>
+  </si>
+  <si>
+    <t>PSC Annual Report Application. Release 2026.04. Pacific Salmon Commission. [Updated 2026 Apr 17; accessed 2026 Apr 20]. https://www.psc1.shinyapps.io/PSC_Annual_Fraser/</t>
+  </si>
+  <si>
+    <t>PSC_20260417</t>
   </si>
 </sst>
 </file>
@@ -772,7 +778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24029AEC-6FE5-6340-8374-FCF69BAFD37B}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
@@ -1012,6 +1018,14 @@
         <v>57</v>
       </c>
     </row>
+    <row r="30" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B26">
     <sortCondition ref="A1:A26"/>

</xml_diff>

<commit_message>
Update Yakoun and Skeena data sources
</commit_message>
<xml_diff>
--- a/data/data-sources_2026.xlsx
+++ b/data/data-sources_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hhunter\Documents\state-of-salmon\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9E9979-450E-4206-A7E7-96EA70A458B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C179E800-FB3C-4E48-822F-39402048214C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
+    <workbookView xWindow="-15525" yWindow="-18120" windowWidth="25440" windowHeight="15270" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -272,20 +272,32 @@
     <t>ProvBC_20250903</t>
   </si>
   <si>
-    <t>Province of British Columbia. 2023. Estimated Escapement of Skeena Summer Steelhead at the Tyee Test Fishery, 1956 - 2024 - All Years to Sept 2, 2025. Provided to Pacific Salmon Foundation by Kenji Miyazaki on September 3, 2025.</t>
-  </si>
-  <si>
     <t>Spoljaric_20260409</t>
   </si>
   <si>
     <t>Spoljaric, Mark. 2026. Summary of Yakoun Chinook escapement estimates, 2021 - 2025. Provided to Pacific Salmon Foundation by Mark Spoljaric (Haida Fisheries Program) on April 9, 2026.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Province of British Columbia. 2025. Estimated Escapement of Skeena Summer Steelhead at the Tyee Test Fishery, 1956 - 2024 - All Years to Sept 2, 2025. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Provided to Pacific Salmon Foundation by Kenji Miyazaki on September 3, 2025.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -330,6 +342,13 @@
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -989,15 +1008,15 @@
         <v>54</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A29" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="14" t="s">
         <v>56</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Delete old data source
</commit_message>
<xml_diff>
--- a/data/data-sources_2026.xlsx
+++ b/data/data-sources_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hhunter\Documents\state-of-salmon\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C179E800-FB3C-4E48-822F-39402048214C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD77B9CF-2090-4FD8-9663-92949A373320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15525" yWindow="-18120" windowWidth="25440" windowHeight="15270" xr2:uid="{E96813F5-1777-F041-8F52-E9C9A952FEDD}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>source_id</t>
   </si>
@@ -127,12 +127,6 @@
   </si>
   <si>
     <t>CarrHarris_20250724</t>
-  </si>
-  <si>
-    <t>ProvBC_20240929</t>
-  </si>
-  <si>
-    <t>Province of British Columbia. 2023. Estimated Escapement of Skeena Summer Steelhead at the Tyee Test Fishery, 1956 - 2024 - All Years to Aug 29, 2024.</t>
   </si>
   <si>
     <t>Brown_20250703</t>
@@ -279,7 +273,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Province of British Columbia. 2025. Estimated Escapement of Skeena Summer Steelhead at the Tyee Test Fishery, 1956 - 2024 - All Years to Sept 2, 2025. </t>
+      <t xml:space="preserve">Province of British Columbia. 2025. Estimated Escapement of Skeena Summer Steelhead at the Tyee Test Fishery, 1956 - 2025 - All Years to Sept 2, 2025. </t>
     </r>
     <r>
       <rPr>
@@ -779,7 +773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24029AEC-6FE5-6340-8374-FCF69BAFD37B}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.69921875" customWidth="1"/>
@@ -796,27 +790,27 @@
     </row>
     <row r="2" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
@@ -824,7 +818,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
@@ -837,34 +831,34 @@
     </row>
     <row r="7" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="62.4" x14ac:dyDescent="0.3">
@@ -885,42 +879,42 @@
     </row>
     <row r="13" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
@@ -933,95 +927,87 @@
     </row>
     <row r="19" spans="1:2" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>12</v>
-      </c>
-      <c r="B26" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="s">
+    <row r="26" spans="1:2" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="12" t="s">
-        <v>53</v>
+      <c r="B27" s="14" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>56</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B26">
-    <sortCondition ref="A1:A26"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B25">
+    <sortCondition ref="A1:A25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>